<commit_message>
update 7 invoice templates to latest user source (2026-08-14): 中运通达174→38行 etc
</commit_message>
<xml_diff>
--- a/templates/tpl_msecxi8m_ulv90a.xlsx
+++ b/templates/tpl_msecxi8m_ulv90a.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="12935"/>
+    <workbookView windowWidth="22188" windowHeight="10055"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -196,7 +196,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>L/C No.:</t>
   </si>
@@ -267,7 +267,7 @@
     <t>材质</t>
   </si>
   <si>
-    <t>规格/尺寸</t>
+    <t>纸箱规格/尺寸</t>
   </si>
   <si>
     <t>品牌类型</t>
@@ -298,6 +298,9 @@
   </si>
   <si>
     <t>USAGE</t>
+  </si>
+  <si>
+    <t>SKU</t>
   </si>
   <si>
     <t>BRAND</t>
@@ -1255,7 +1258,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1291,7 +1294,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1327,7 +1330,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1363,7 +1366,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1399,7 +1402,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1435,7 +1438,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1471,7 +1474,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1507,7 +1510,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1543,7 +1546,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1579,7 +1582,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1615,7 +1618,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1651,7 +1654,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1687,7 +1690,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1723,7 +1726,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1759,7 +1762,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1795,7 +1798,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1831,7 +1834,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1867,7 +1870,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1903,7 +1906,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1939,7 +1942,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1975,7 +1978,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2011,7 +2014,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2047,7 +2050,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2083,7 +2086,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2119,7 +2122,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2155,7 +2158,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2191,7 +2194,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2227,7 +2230,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2263,7 +2266,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2299,7 +2302,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2335,7 +2338,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2371,7 +2374,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2407,7 +2410,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2443,7 +2446,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2479,7 +2482,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2515,7 +2518,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2551,7 +2554,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2587,7 +2590,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2623,7 +2626,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2659,7 +2662,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2695,7 +2698,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2731,7 +2734,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2767,7 +2770,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2803,7 +2806,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2839,7 +2842,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2875,7 +2878,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2911,7 +2914,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2947,7 +2950,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2983,7 +2986,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3019,7 +3022,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3055,7 +3058,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3091,7 +3094,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3127,7 +3130,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3163,7 +3166,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3199,7 +3202,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3235,7 +3238,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3271,7 +3274,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3307,7 +3310,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3343,7 +3346,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3379,7 +3382,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3415,7 +3418,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3451,7 +3454,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3487,7 +3490,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="0"/>
+          <a:off x="13536930" y="0"/>
           <a:ext cx="304800" cy="305435"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3523,7 +3526,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="3481070"/>
+          <a:off x="13536930" y="2716530"/>
           <a:ext cx="304800" cy="304800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3559,7 +3562,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13363575" y="3481070"/>
+          <a:off x="13536930" y="2716530"/>
           <a:ext cx="304800" cy="304800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3838,11 +3841,12 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="19.25" customWidth="1"/>
-    <col min="2" max="2" width="10.125" customWidth="1"/>
-    <col min="3" max="3" width="12.5" customWidth="1"/>
+    <col min="2" max="2" width="10.4" customWidth="1"/>
+    <col min="3" max="3" width="14.9" customWidth="1"/>
     <col min="4" max="4" width="12.125" customWidth="1"/>
     <col min="5" max="5" width="10.625" customWidth="1"/>
-    <col min="6" max="7" width="10.5" customWidth="1"/>
+    <col min="6" max="6" width="10.1" customWidth="1"/>
+    <col min="7" max="7" width="10.5" customWidth="1"/>
     <col min="8" max="8" width="11.75" customWidth="1"/>
     <col min="9" max="9" width="8.875" customWidth="1"/>
     <col min="10" max="10" width="17.25" customWidth="1"/>
@@ -3909,7 +3913,7 @@
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
     </row>
-    <row r="6" ht="20.1" customHeight="1" spans="1:15">
+    <row r="6" ht="27" customHeight="1" spans="1:15">
       <c r="A6" s="8" t="s">
         <v>6</v>
       </c>
@@ -3956,7 +3960,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" ht="20.1" customHeight="1" spans="1:15">
+    <row r="7" ht="27" customHeight="1" spans="1:15">
       <c r="A7" s="12" t="s">
         <v>21</v>
       </c>
@@ -3984,18 +3988,20 @@
       <c r="I7" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="10"/>
-      <c r="K7" s="8" t="s">
+      <c r="J7" s="10" t="s">
         <v>29</v>
       </c>
+      <c r="K7" s="8" t="s">
+        <v>30</v>
+      </c>
       <c r="L7" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
       <c r="O7" s="16"/>
     </row>
-    <row r="8" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="8" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -4012,7 +4018,7 @@
       <c r="N8" s="21"/>
       <c r="O8" s="22"/>
     </row>
-    <row r="9" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="9" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -4029,7 +4035,7 @@
       <c r="N9" s="21"/>
       <c r="O9" s="22"/>
     </row>
-    <row r="10" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="10" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -4046,7 +4052,7 @@
       <c r="N10" s="21"/>
       <c r="O10" s="23"/>
     </row>
-    <row r="11" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="11" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A11" s="17"/>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -4063,7 +4069,7 @@
       <c r="N11" s="21"/>
       <c r="O11" s="23"/>
     </row>
-    <row r="12" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="12" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -4080,7 +4086,7 @@
       <c r="N12" s="21"/>
       <c r="O12" s="23"/>
     </row>
-    <row r="13" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="13" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A13" s="17"/>
       <c r="B13" s="17"/>
       <c r="C13" s="17"/>
@@ -4097,7 +4103,7 @@
       <c r="N13" s="21"/>
       <c r="O13" s="23"/>
     </row>
-    <row r="14" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="14" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A14" s="17"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -4114,7 +4120,7 @@
       <c r="N14" s="21"/>
       <c r="O14" s="23"/>
     </row>
-    <row r="15" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="15" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A15" s="17"/>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -4131,7 +4137,7 @@
       <c r="N15" s="21"/>
       <c r="O15" s="23"/>
     </row>
-    <row r="16" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="16" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A16" s="17"/>
       <c r="B16" s="17"/>
       <c r="C16" s="17"/>
@@ -4148,7 +4154,7 @@
       <c r="N16" s="21"/>
       <c r="O16" s="23"/>
     </row>
-    <row r="17" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="17" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A17" s="17"/>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -4165,7 +4171,7 @@
       <c r="N17" s="21"/>
       <c r="O17" s="23"/>
     </row>
-    <row r="18" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="18" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A18" s="17"/>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
@@ -4182,7 +4188,7 @@
       <c r="N18" s="21"/>
       <c r="O18" s="23"/>
     </row>
-    <row r="19" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="19" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A19" s="17"/>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
@@ -4199,7 +4205,7 @@
       <c r="N19" s="21"/>
       <c r="O19" s="23"/>
     </row>
-    <row r="20" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="20" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A20" s="17"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -4216,7 +4222,7 @@
       <c r="N20" s="21"/>
       <c r="O20" s="23"/>
     </row>
-    <row r="21" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="21" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A21" s="17"/>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
@@ -4233,7 +4239,7 @@
       <c r="N21" s="21"/>
       <c r="O21" s="23"/>
     </row>
-    <row r="22" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="22" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A22" s="17"/>
       <c r="B22" s="17"/>
       <c r="C22" s="17"/>
@@ -4250,7 +4256,7 @@
       <c r="N22" s="21"/>
       <c r="O22" s="23"/>
     </row>
-    <row r="23" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="23" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A23" s="17"/>
       <c r="B23" s="17"/>
       <c r="C23" s="17"/>
@@ -4267,7 +4273,7 @@
       <c r="N23" s="21"/>
       <c r="O23" s="23"/>
     </row>
-    <row r="24" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="24" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A24" s="17"/>
       <c r="B24" s="17"/>
       <c r="C24" s="17"/>
@@ -4284,7 +4290,7 @@
       <c r="N24" s="21"/>
       <c r="O24" s="23"/>
     </row>
-    <row r="25" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="25" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A25" s="17"/>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -4301,7 +4307,7 @@
       <c r="N25" s="21"/>
       <c r="O25" s="23"/>
     </row>
-    <row r="26" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="26" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A26" s="17"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
@@ -4318,7 +4324,7 @@
       <c r="N26" s="21"/>
       <c r="O26" s="23"/>
     </row>
-    <row r="27" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="27" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A27" s="17"/>
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
@@ -4335,7 +4341,7 @@
       <c r="N27" s="21"/>
       <c r="O27" s="23"/>
     </row>
-    <row r="28" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="28" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A28" s="17"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -4352,7 +4358,7 @@
       <c r="N28" s="21"/>
       <c r="O28" s="23"/>
     </row>
-    <row r="29" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="29" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A29" s="17"/>
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>
@@ -4369,7 +4375,7 @@
       <c r="N29" s="21"/>
       <c r="O29" s="23"/>
     </row>
-    <row r="30" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="30" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A30" s="17"/>
       <c r="B30" s="17"/>
       <c r="C30" s="17"/>
@@ -4386,7 +4392,7 @@
       <c r="N30" s="21"/>
       <c r="O30" s="23"/>
     </row>
-    <row r="31" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="31" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A31" s="17"/>
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
@@ -4403,7 +4409,7 @@
       <c r="N31" s="21"/>
       <c r="O31" s="23"/>
     </row>
-    <row r="32" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="32" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A32" s="17"/>
       <c r="B32" s="17"/>
       <c r="C32" s="17"/>
@@ -4420,7 +4426,7 @@
       <c r="N32" s="21"/>
       <c r="O32" s="23"/>
     </row>
-    <row r="33" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="33" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A33" s="17"/>
       <c r="B33" s="17"/>
       <c r="C33" s="17"/>
@@ -4437,7 +4443,7 @@
       <c r="N33" s="21"/>
       <c r="O33" s="23"/>
     </row>
-    <row r="34" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="34" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A34" s="17"/>
       <c r="B34" s="17"/>
       <c r="C34" s="17"/>
@@ -4454,7 +4460,7 @@
       <c r="N34" s="21"/>
       <c r="O34" s="23"/>
     </row>
-    <row r="35" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="35" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A35" s="17"/>
       <c r="B35" s="17"/>
       <c r="C35" s="17"/>
@@ -4471,7 +4477,7 @@
       <c r="N35" s="21"/>
       <c r="O35" s="23"/>
     </row>
-    <row r="36" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="36" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A36" s="17"/>
       <c r="B36" s="17"/>
       <c r="C36" s="17"/>
@@ -4488,7 +4494,7 @@
       <c r="N36" s="21"/>
       <c r="O36" s="23"/>
     </row>
-    <row r="37" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="37" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A37" s="17"/>
       <c r="B37" s="17"/>
       <c r="C37" s="17"/>
@@ -4505,7 +4511,7 @@
       <c r="N37" s="21"/>
       <c r="O37" s="23"/>
     </row>
-    <row r="38" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="38" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A38" s="17"/>
       <c r="B38" s="17"/>
       <c r="C38" s="17"/>
@@ -4522,7 +4528,7 @@
       <c r="N38" s="21"/>
       <c r="O38" s="23"/>
     </row>
-    <row r="39" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="39" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A39" s="17"/>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -4539,7 +4545,7 @@
       <c r="N39" s="21"/>
       <c r="O39" s="23"/>
     </row>
-    <row r="40" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="40" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A40" s="17"/>
       <c r="B40" s="17"/>
       <c r="C40" s="17"/>
@@ -4556,7 +4562,7 @@
       <c r="N40" s="21"/>
       <c r="O40" s="23"/>
     </row>
-    <row r="41" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="41" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A41" s="17"/>
       <c r="B41" s="17"/>
       <c r="C41" s="17"/>
@@ -4573,7 +4579,7 @@
       <c r="N41" s="21"/>
       <c r="O41" s="23"/>
     </row>
-    <row r="42" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="42" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A42" s="17"/>
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
@@ -4590,7 +4596,7 @@
       <c r="N42" s="21"/>
       <c r="O42" s="23"/>
     </row>
-    <row r="43" s="1" customFormat="1" ht="62" customHeight="1" spans="1:15">
+    <row r="43" s="1" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A43" s="17"/>
       <c r="B43" s="17"/>
       <c r="C43" s="17"/>
@@ -4653,9 +4659,6 @@
     <row r="84" s="2" customFormat="1"/>
     <row r="85" s="2" customFormat="1"/>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A7:O44" etc:filterBottomFollowUsedRange="0">
-    <extLst/>
-  </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B1:G2"/>

</xml_diff>